<commit_message>
Adding intermediate edits for various projects
</commit_message>
<xml_diff>
--- a/LSPC/Weather_File_Generation/inputs/Project_Control_Navarro.xlsx
+++ b/LSPC/Weather_File_Generation/inputs/Project_Control_Navarro.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCB112C-4FFE-4142-BC41-EBF00417E1C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
@@ -9146,6 +9146,42 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="84c16208-172a-4eaa-b33e-1408ce0b909e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <LastModifiedBy xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </LastModifiedBy>
+    <LastModifiedOn xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"Blank Document","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AD1B9453B0FD26428396C40DDB69C7F0" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7ae69fa2ec7ba05b1cd5ad5facbfed2a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="04ff8bd0-14ef-4472-a603-3a4b6f9fed19" xmlns:ns3="84c16208-172a-4eaa-b33e-1408ce0b909e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="593a7e08a14a0b523a37a1b36e06b6ea" ns2:_="" ns3:_="">
     <xsd:import namespace="04ff8bd0-14ef-4472-a603-3a4b6f9fed19"/>
@@ -9378,43 +9414,44 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"Blank Document","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41E32FE7-C838-46D6-8359-8A7BBC9B619E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A7D180A-E261-4A2D-8CBC-AEEBF9B497B3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="84c16208-172a-4eaa-b33e-1408ce0b909e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="04ff8bd0-14ef-4472-a603-3a4b6f9fed19"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="84c16208-172a-4eaa-b33e-1408ce0b909e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <LastModifiedBy xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </LastModifiedBy>
-    <LastModifiedOn xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06124858-FF52-43B6-9F5F-14F707108C35}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{43BD7F1F-596C-48D7-B49B-C059BD9AD9F3}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C924A6F-1A37-48C2-B047-4F31E4508879}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9433,43 +9470,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{43BD7F1F-596C-48D7-B49B-C059BD9AD9F3}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06124858-FF52-43B6-9F5F-14F707108C35}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A7D180A-E261-4A2D-8CBC-AEEBF9B497B3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="84c16208-172a-4eaa-b33e-1408ce0b909e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="04ff8bd0-14ef-4472-a603-3a4b6f9fed19"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41E32FE7-C838-46D6-8359-8A7BBC9B619E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0bb6ca0c-ccb3-428b-9d5f-a9c60cad6645}" enabled="1" method="Standard" siteId="{fe186a25-7d49-41e6-9941-05d2281d36c1}" contentBits="0" removed="0"/>

</xml_diff>